<commit_message>
Techreview 2 doc finish
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HydrogenRb\HydrogenRb\Work\tech\Agent\8_14\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE3EE6C-1DB6-4086-81D3-FF42F01150E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D08A88B-8B27-4A63-9A0B-28602DE5D357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="集成" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="62">
   <si>
     <t>分类</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -202,6 +202,78 @@
   </si>
   <si>
     <t>ahb_test_6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test_bus_{{i}}_dat</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test_bus_{{i}}_ready</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test_bus_{{i}}_valid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test_bus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>155、…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>`DW_{{i}}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>i的范围是{sig1,sig2,sig3}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>i的列表{sig1,sig2,sig3}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>i的列表是{sig1,sig2,sig3}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CHI_interface</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chi_if_risc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sky_cs_if.mst</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dyadic array</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>array</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>`LANE_NUM * `Test</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3*100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>`LANE_NUM * `Test_size</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -245,12 +317,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -531,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:Y18"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" width="9.33203125" customWidth="1"/>
@@ -969,7 +1040,21 @@
       <c r="G9" t="s">
         <v>5</v>
       </c>
-      <c r="I9" s="2"/>
+      <c r="I9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J9" t="s">
+        <v>58</v>
+      </c>
+      <c r="K9" t="s">
+        <v>20</v>
+      </c>
+      <c r="L9" t="s">
+        <v>58</v>
+      </c>
+      <c r="M9" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A10" s="1"/>
@@ -979,7 +1064,6 @@
       <c r="C10" t="s">
         <v>5</v>
       </c>
-      <c r="I10" s="2"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
@@ -1004,22 +1088,105 @@
         <v>5</v>
       </c>
     </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A15" s="1"/>
+      <c r="B15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A16" s="1"/>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="I3:I8"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
     <mergeCell ref="P1:Q1"/>
     <mergeCell ref="O3:O8"/>
     <mergeCell ref="T1:U1"/>
     <mergeCell ref="S3:S8"/>
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="W3:W8"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="I3:I8"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A6:A10"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1028,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{202D62A6-CB45-4A21-B036-6EE2427F8DDC}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.4">
@@ -1220,7 +1387,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A17" s="1"/>
       <c r="B17" t="s">
         <v>25</v>
@@ -1232,7 +1399,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A18" s="1"/>
       <c r="B18" t="s">
         <v>26</v>
@@ -1244,7 +1411,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A19" s="1"/>
       <c r="B19" t="s">
         <v>43</v>
@@ -1256,11 +1423,70 @@
         <v>20</v>
       </c>
     </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E21" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" t="s">
+        <v>5</v>
+      </c>
+      <c r="I21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A22" s="1"/>
+      <c r="B22" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A23" s="1"/>
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" t="s">
+        <v>55</v>
+      </c>
+      <c r="F25" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="A14:A19"/>
+    <mergeCell ref="A21:A23"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1269,7 +1495,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1F3E398-7E0A-4C3A-A273-DA12B1D3ED24}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.4">
@@ -1364,9 +1590,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A8" s="2"/>
-    </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>12</v>
@@ -1458,7 +1681,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
@@ -1472,7 +1695,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A19" s="1"/>
       <c r="B19" t="s">
         <v>15</v>
@@ -1484,7 +1707,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A20" s="1"/>
       <c r="B20" t="s">
         <v>16</v>
@@ -1496,7 +1719,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A21" s="1"/>
       <c r="B21" t="s">
         <v>17</v>
@@ -1508,7 +1731,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A22" s="1"/>
       <c r="B22" t="s">
         <v>18</v>
@@ -1520,7 +1743,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A23" s="1"/>
       <c r="B23" t="s">
         <v>19</v>
@@ -1532,12 +1755,88 @@
         <v>20</v>
       </c>
     </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A25" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25" t="s">
+        <v>5</v>
+      </c>
+      <c r="I25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A26" s="1"/>
+      <c r="B26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A27" s="1"/>
+      <c r="B27" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" t="s">
+        <v>54</v>
+      </c>
+      <c r="D29" t="s">
+        <v>55</v>
+      </c>
+      <c r="F29" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" t="s">
+        <v>61</v>
+      </c>
+      <c r="E31" t="s">
+        <v>60</v>
+      </c>
+      <c r="F31" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A11:A16"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A18:A23"/>
+    <mergeCell ref="A25:A27"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1546,7 +1845,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F2DC5A-AAE7-49CB-BE38-CB832B2EDA63}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.4">
@@ -1759,7 +2058,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A17" s="1"/>
       <c r="B17" t="s">
         <v>18</v>
@@ -1771,7 +2070,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A18" s="1"/>
       <c r="B18" t="s">
         <v>19</v>
@@ -1783,7 +2082,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
@@ -1797,7 +2096,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A21" s="1"/>
       <c r="B21" t="s">
         <v>23</v>
@@ -1809,7 +2108,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A22" s="1"/>
       <c r="B22" t="s">
         <v>24</v>
@@ -1821,7 +2120,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A23" s="1"/>
       <c r="B23" t="s">
         <v>25</v>
@@ -1833,7 +2132,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
       <c r="B24" t="s">
         <v>26</v>
@@ -1845,7 +2144,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A25" s="1"/>
       <c r="B25" t="s">
         <v>26</v>
@@ -1857,12 +2156,74 @@
         <v>20</v>
       </c>
     </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" t="s">
+        <v>49</v>
+      </c>
+      <c r="E27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" t="s">
+        <v>5</v>
+      </c>
+      <c r="I27" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A28" s="1"/>
+      <c r="B28" t="s">
+        <v>45</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A29" s="1"/>
+      <c r="B29" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" t="s">
+        <v>59</v>
+      </c>
+      <c r="E31" t="s">
+        <v>60</v>
+      </c>
+      <c r="F31" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A20:A25"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A13:A18"/>
     <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A27:A29"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add multi page function
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HydrogenRb\HydrogenRb\Work\tech\Agent\8_14\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F84DD9-800C-4613-9469-874CD649B169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EFE3D5E-346B-4B90-8671-263B0E1804CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="集成" sheetId="1" r:id="rId1"/>
-    <sheet name="RISCV_TOP" sheetId="2" r:id="rId2"/>
-    <sheet name="RISCV_CORE_TEST" sheetId="3" r:id="rId3"/>
-    <sheet name="MEM_PHY" sheetId="4" r:id="rId4"/>
+    <sheet name="集成_RISCV_TOP" sheetId="1" r:id="rId1"/>
+    <sheet name="集成_RISCV_CORE_TEST" sheetId="5" r:id="rId2"/>
+    <sheet name="RISCV_TOP" sheetId="2" r:id="rId3"/>
+    <sheet name="RISCV_CORE_TEST" sheetId="3" r:id="rId4"/>
+    <sheet name="MEM_PHY" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="69">
   <si>
     <t>分类</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1247,6 +1248,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="O3:O8"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="S3:S8"/>
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="W3:W8"/>
     <mergeCell ref="A3:A4"/>
@@ -1258,11 +1264,6 @@
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="F1:G1"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="O3:O8"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="S3:S8"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1270,6 +1271,647 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C48CD3-93F9-434D-BA45-1CF2A2B42A74}">
+  <dimension ref="A1:Y22"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="3" max="3" width="9.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="10" max="10" width="10.1328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" s="1"/>
+      <c r="J1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1" s="1"/>
+      <c r="P1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" s="1"/>
+      <c r="T1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="U1" s="1"/>
+      <c r="X1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y1" s="1"/>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O2" t="s">
+        <v>0</v>
+      </c>
+      <c r="P2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>2</v>
+      </c>
+      <c r="S2" t="s">
+        <v>0</v>
+      </c>
+      <c r="T2" t="s">
+        <v>1</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2</v>
+      </c>
+      <c r="W2" t="s">
+        <v>0</v>
+      </c>
+      <c r="X2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>5</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="T3" t="s">
+        <v>21</v>
+      </c>
+      <c r="U3" t="s">
+        <v>5</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A4" s="1"/>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" t="s">
+        <v>20</v>
+      </c>
+      <c r="O4" s="1"/>
+      <c r="P4" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>5</v>
+      </c>
+      <c r="S4" s="1"/>
+      <c r="T4" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" t="s">
+        <v>5</v>
+      </c>
+      <c r="W4" s="1"/>
+      <c r="X4" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="I5" s="1"/>
+      <c r="J5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" t="s">
+        <v>5</v>
+      </c>
+      <c r="O5" s="1"/>
+      <c r="P5" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>20</v>
+      </c>
+      <c r="S5" s="1"/>
+      <c r="T5" t="s">
+        <v>24</v>
+      </c>
+      <c r="U5" t="s">
+        <v>20</v>
+      </c>
+      <c r="W5" s="1"/>
+      <c r="X5" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" t="s">
+        <v>20</v>
+      </c>
+      <c r="L6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" t="s">
+        <v>5</v>
+      </c>
+      <c r="O6" s="1"/>
+      <c r="P6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>20</v>
+      </c>
+      <c r="S6" s="1"/>
+      <c r="T6" t="s">
+        <v>25</v>
+      </c>
+      <c r="U6" t="s">
+        <v>20</v>
+      </c>
+      <c r="W6" s="1"/>
+      <c r="X6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A7" s="1"/>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" t="s">
+        <v>18</v>
+      </c>
+      <c r="M7" t="s">
+        <v>5</v>
+      </c>
+      <c r="O7" s="1"/>
+      <c r="P7" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>20</v>
+      </c>
+      <c r="S7" s="1"/>
+      <c r="T7" t="s">
+        <v>26</v>
+      </c>
+      <c r="U7" t="s">
+        <v>20</v>
+      </c>
+      <c r="W7" s="1"/>
+      <c r="X7" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A8" s="1"/>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="J8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" t="s">
+        <v>20</v>
+      </c>
+      <c r="L8" t="s">
+        <v>19</v>
+      </c>
+      <c r="M8" t="s">
+        <v>5</v>
+      </c>
+      <c r="O8" s="1"/>
+      <c r="P8" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>20</v>
+      </c>
+      <c r="S8" s="1"/>
+      <c r="T8" t="s">
+        <v>26</v>
+      </c>
+      <c r="U8" t="s">
+        <v>20</v>
+      </c>
+      <c r="W8" s="1"/>
+      <c r="X8" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A9" s="1"/>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>5</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" t="s">
+        <v>5</v>
+      </c>
+      <c r="I9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J9" t="s">
+        <v>58</v>
+      </c>
+      <c r="K9" t="s">
+        <v>20</v>
+      </c>
+      <c r="L9" t="s">
+        <v>58</v>
+      </c>
+      <c r="M9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A10" s="1"/>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A15" s="1"/>
+      <c r="B15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A16" s="1"/>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A20" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A21" s="1"/>
+      <c r="B21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A22" s="1"/>
+      <c r="B22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="I3:I8"/>
+    <mergeCell ref="O3:O8"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="W3:W8"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="P1:Q1"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{202D62A6-CB45-4A21-B036-6EE2427F8DDC}">
   <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
@@ -1605,7 +2247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1F3E398-7E0A-4C3A-A273-DA12B1D3ED24}">
   <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
@@ -1994,7 +2636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F2DC5A-AAE7-49CB-BE38-CB832B2EDA63}">
   <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>

</xml_diff>